<commit_message>
auto: 작업 자동 저장 2026-07-30 09:26
Co-Authored-By: Claude Fable 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/eval-runner/orchestrator/data/RV2/06_calibration/RV2_judge_캘리브레이션_판정30_v1_0.xlsx
+++ b/eval-runner/orchestrator/data/RV2/06_calibration/RV2_judge_캘리브레이션_판정30_v1_0.xlsx
@@ -491,8 +491,11 @@
           <t>'도입 확대'와 '책임 강화' 두 측면을 모두 포함하면 정답</t>
         </is>
       </c>
-      <c r="F2" t="inlineStr"/>
-      <c r="G2" t="inlineStr"/>
+      <c r="F2" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -521,8 +524,11 @@
           <t>'작동 방식이 근본적으로 다르다'는 취지를 포함하면 정답</t>
         </is>
       </c>
-      <c r="F3" t="inlineStr"/>
-      <c r="G3" t="inlineStr"/>
+      <c r="F3" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -551,8 +557,11 @@
           <t>필수 요소(고급 암호화 프로토콜, 이중 인증) 모두 포함하고 출처 일치</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr"/>
-      <c r="G4" t="inlineStr"/>
+      <c r="F4" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -581,8 +590,11 @@
           <t>채널 수=동시 접속 가능한 기기 수, 세션 수=한 사람이 동시 제어 가능한 기기 수라는 두 개념 구분이 모두 포함되면 정답 처리한다.</t>
         </is>
       </c>
-      <c r="F5" t="inlineStr"/>
-      <c r="G5" t="inlineStr"/>
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -611,8 +623,11 @@
           <t>인터넷 연결 조건과 사무실 PC 원격 접속 가능을 모두 언급</t>
         </is>
       </c>
-      <c r="F6" t="inlineStr"/>
-      <c r="G6" t="inlineStr"/>
+      <c r="F6" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -641,8 +656,11 @@
           <t>OTP와 2단계 보안 설정을 정답에 포함</t>
         </is>
       </c>
-      <c r="F7" t="inlineStr"/>
-      <c r="G7" t="inlineStr"/>
+      <c r="F7" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -671,8 +689,11 @@
           <t>화면 가림과 정보 노출 방지를 정답에 포함</t>
         </is>
       </c>
-      <c r="F8" t="inlineStr"/>
-      <c r="G8" t="inlineStr"/>
+      <c r="F8" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -701,8 +722,11 @@
           <t>PC/사용자를 그룹 단위로 관리하는 기능을 제공한다는 점을 명시</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr"/>
-      <c r="G9" t="inlineStr"/>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -731,8 +755,11 @@
           <t>'여러 대의 모니터(멀티/듀얼)'와 '제어 가능'을 포함하면 정답.</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr"/>
-      <c r="G10" t="inlineStr"/>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -761,8 +788,11 @@
           <t>SI 업체·외주 개발 기업·프리랜서 개발자 세 대상을 모두 언급</t>
         </is>
       </c>
-      <c r="F11" t="inlineStr"/>
-      <c r="G11" t="inlineStr"/>
+      <c r="F11" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -791,8 +821,11 @@
           <t>필수 요소 'MFA', 'RBAC', '감사 로그'가 모두 포함되면 정답 처리한다.</t>
         </is>
       </c>
-      <c r="F12" t="inlineStr"/>
-      <c r="G12" t="inlineStr"/>
+      <c r="F12" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -821,8 +854,11 @@
           <t>외부 인력의 작업 과정을 투명하게 감독한다는 취지를 언급</t>
         </is>
       </c>
-      <c r="F13" t="inlineStr"/>
-      <c r="G13" t="inlineStr"/>
+      <c r="F13" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -851,8 +887,11 @@
           <t>구글 SSO 로그인과 안드로이드 원격제어 호환성 강화를 모두 언급</t>
         </is>
       </c>
-      <c r="F14" t="inlineStr"/>
-      <c r="G14" t="inlineStr"/>
+      <c r="F14" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -881,8 +920,11 @@
           <t>'VDI는 서버 증설 필요', '리모트뷰는 라이선스 추가만으로 해결' 두 대비를 모두 언급하면 정답.</t>
         </is>
       </c>
-      <c r="F15" t="inlineStr"/>
-      <c r="G15" t="inlineStr"/>
+      <c r="F15" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -911,8 +953,11 @@
           <t>KVM과 달리 단순 화면 공유에 그치지 않는다는 차별점을 포함</t>
         </is>
       </c>
-      <c r="F16" t="inlineStr"/>
-      <c r="G16" t="inlineStr"/>
+      <c r="F16" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -941,8 +986,11 @@
           <t>필수 요소 'IT-OT'와 '하나의 플랫폼'이 모두 포함되면 정답 처리한다.</t>
         </is>
       </c>
-      <c r="F17" t="inlineStr"/>
-      <c r="G17" t="inlineStr"/>
+      <c r="F17" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -971,8 +1019,11 @@
           <t>대한민국 본사에서 직접 기술지원을 제공한다는 점을 명시</t>
         </is>
       </c>
-      <c r="F18" t="inlineStr"/>
-      <c r="G18" t="inlineStr"/>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -1001,8 +1052,11 @@
           <t>90%를 정확히 제시하고 재택근무 비율(원격근무 인프라 성숙) 맥락을 포함하면 정답</t>
         </is>
       </c>
-      <c r="F19" t="inlineStr"/>
-      <c r="G19" t="inlineStr"/>
+      <c r="F19" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -1031,8 +1085,11 @@
           <t>RDP 설정·보안 취약점과 무료 툴 기능 한계를 모두 포함</t>
         </is>
       </c>
-      <c r="F20" t="inlineStr"/>
-      <c r="G20" t="inlineStr"/>
+      <c r="F20" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -1061,8 +1118,11 @@
           <t>소프트웨어 무설치와 하드웨어 기반 제어 두 요소를 모두 포함</t>
         </is>
       </c>
-      <c r="F21" t="inlineStr"/>
-      <c r="G21" t="inlineStr"/>
+      <c r="F21" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -1091,8 +1151,11 @@
           <t>촬영 시 식별·추적이 모두 불가능하다는 사실을 명시</t>
         </is>
       </c>
-      <c r="F22" t="inlineStr"/>
-      <c r="G22" t="inlineStr"/>
+      <c r="F22" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -1121,8 +1184,11 @@
           <t>O/S 보안 패치 점검과 백신 업데이트 상태 확인 두 요소를 모두 포함</t>
         </is>
       </c>
-      <c r="F23" t="inlineStr"/>
-      <c r="G23" t="inlineStr"/>
+      <c r="F23" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -1151,8 +1217,11 @@
           <t>OS 무관과 HDMI·DVI·VGA 등 포트 지원을 함께 명시</t>
         </is>
       </c>
-      <c r="F24" t="inlineStr"/>
-      <c r="G24" t="inlineStr"/>
+      <c r="F24" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -1181,8 +1250,11 @@
           <t>IT 인력 부족·24시간 상주 어려움과 최소 인력 최대 효율을 모두 포함</t>
         </is>
       </c>
-      <c r="F25" t="inlineStr"/>
-      <c r="G25" t="inlineStr"/>
+      <c r="F25" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -1211,8 +1283,11 @@
           <t>'KVM 스위치의 랙 단위 제약 극복'과 '다양한 기기에 유연한 연결' 두 요소를 모두 언급하면 정답.</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr"/>
-      <c r="G26" t="inlineStr"/>
+      <c r="F26" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -1241,8 +1316,11 @@
           <t>'프로세스/시스템/앱 설치 정보 확인'과 '재실행·앱 삭제 가능'을 모두 언급하면 정답.</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr"/>
-      <c r="G27" t="inlineStr"/>
+      <c r="F27" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -1271,8 +1349,11 @@
           <t>60FPS와 끊김 없는 제어 품질을 정답에 포함</t>
         </is>
       </c>
-      <c r="F28" t="inlineStr"/>
-      <c r="G28" t="inlineStr"/>
+      <c r="F28" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -1301,8 +1382,11 @@
           <t>'간단한 인증만으로' 체험이 가능하다는 취지가 포함되어야 함</t>
         </is>
       </c>
-      <c r="F29" t="inlineStr"/>
-      <c r="G29" t="inlineStr"/>
+      <c r="F29" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -1331,8 +1415,11 @@
           <t>'10대 이하 기기'와 '실속형(적합)'을 포함하면 정답.</t>
         </is>
       </c>
-      <c r="F30" t="inlineStr"/>
-      <c r="G30" t="inlineStr"/>
+      <c r="F30" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -1361,8 +1448,11 @@
           <t>정답에 네 개 제품명(리모트뷰·스플래시탑·애니데스크·팀뷰어)이 모두 포함되어야 함.</t>
         </is>
       </c>
-      <c r="F31" t="inlineStr"/>
-      <c r="G31" t="inlineStr"/>
+      <c r="F31" t="inlineStr">
+        <is>
+          <t>합격</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <dataValidations count="1">
@@ -2272,9 +2362,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C2" t="inlineStr"/>
-      <c r="D2" t="inlineStr"/>
-      <c r="E2" t="inlineStr"/>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -2287,9 +2374,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C3" t="inlineStr"/>
-      <c r="D3" t="inlineStr"/>
-      <c r="E3" t="inlineStr"/>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -2302,9 +2386,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C4" t="inlineStr"/>
-      <c r="D4" t="inlineStr"/>
-      <c r="E4" t="inlineStr"/>
     </row>
     <row r="5">
       <c r="A5" t="inlineStr">
@@ -2317,9 +2398,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C5" t="inlineStr"/>
-      <c r="D5" t="inlineStr"/>
-      <c r="E5" t="inlineStr"/>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
@@ -2332,9 +2410,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C6" t="inlineStr"/>
-      <c r="D6" t="inlineStr"/>
-      <c r="E6" t="inlineStr"/>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
@@ -2347,9 +2422,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C7" t="inlineStr"/>
-      <c r="D7" t="inlineStr"/>
-      <c r="E7" t="inlineStr"/>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
@@ -2362,9 +2434,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C8" t="inlineStr"/>
-      <c r="D8" t="inlineStr"/>
-      <c r="E8" t="inlineStr"/>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
@@ -2377,9 +2446,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C9" t="inlineStr"/>
-      <c r="D9" t="inlineStr"/>
-      <c r="E9" t="inlineStr"/>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
@@ -2392,9 +2458,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C10" t="inlineStr"/>
-      <c r="D10" t="inlineStr"/>
-      <c r="E10" t="inlineStr"/>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
@@ -2407,9 +2470,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C11" t="inlineStr"/>
-      <c r="D11" t="inlineStr"/>
-      <c r="E11" t="inlineStr"/>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
@@ -2422,9 +2482,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C12" t="inlineStr"/>
-      <c r="D12" t="inlineStr"/>
-      <c r="E12" t="inlineStr"/>
     </row>
     <row r="13">
       <c r="A13" t="inlineStr">
@@ -2437,9 +2494,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C13" t="inlineStr"/>
-      <c r="D13" t="inlineStr"/>
-      <c r="E13" t="inlineStr"/>
     </row>
     <row r="14">
       <c r="A14" t="inlineStr">
@@ -2452,9 +2506,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C14" t="inlineStr"/>
-      <c r="D14" t="inlineStr"/>
-      <c r="E14" t="inlineStr"/>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
@@ -2467,9 +2518,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C15" t="inlineStr"/>
-      <c r="D15" t="inlineStr"/>
-      <c r="E15" t="inlineStr"/>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
@@ -2482,9 +2530,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C16" t="inlineStr"/>
-      <c r="D16" t="inlineStr"/>
-      <c r="E16" t="inlineStr"/>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
@@ -2497,9 +2542,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C17" t="inlineStr"/>
-      <c r="D17" t="inlineStr"/>
-      <c r="E17" t="inlineStr"/>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
@@ -2512,9 +2554,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C18" t="inlineStr"/>
-      <c r="D18" t="inlineStr"/>
-      <c r="E18" t="inlineStr"/>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
@@ -2527,9 +2566,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C19" t="inlineStr"/>
-      <c r="D19" t="inlineStr"/>
-      <c r="E19" t="inlineStr"/>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
@@ -2542,9 +2578,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr"/>
-      <c r="D20" t="inlineStr"/>
-      <c r="E20" t="inlineStr"/>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
@@ -2557,9 +2590,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr"/>
-      <c r="D21" t="inlineStr"/>
-      <c r="E21" t="inlineStr"/>
     </row>
     <row r="22">
       <c r="A22" t="inlineStr">
@@ -2572,9 +2602,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C22" t="inlineStr"/>
-      <c r="D22" t="inlineStr"/>
-      <c r="E22" t="inlineStr"/>
     </row>
     <row r="23">
       <c r="A23" t="inlineStr">
@@ -2587,9 +2614,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr"/>
-      <c r="D23" t="inlineStr"/>
-      <c r="E23" t="inlineStr"/>
     </row>
     <row r="24">
       <c r="A24" t="inlineStr">
@@ -2602,9 +2626,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C24" t="inlineStr"/>
-      <c r="D24" t="inlineStr"/>
-      <c r="E24" t="inlineStr"/>
     </row>
     <row r="25">
       <c r="A25" t="inlineStr">
@@ -2617,9 +2638,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C25" t="inlineStr"/>
-      <c r="D25" t="inlineStr"/>
-      <c r="E25" t="inlineStr"/>
     </row>
     <row r="26">
       <c r="A26" t="inlineStr">
@@ -2632,9 +2650,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr"/>
-      <c r="D26" t="inlineStr"/>
-      <c r="E26" t="inlineStr"/>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
@@ -2647,9 +2662,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr"/>
-      <c r="D27" t="inlineStr"/>
-      <c r="E27" t="inlineStr"/>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
@@ -2662,9 +2674,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C28" t="inlineStr"/>
-      <c r="D28" t="inlineStr"/>
-      <c r="E28" t="inlineStr"/>
     </row>
     <row r="29">
       <c r="A29" t="inlineStr">
@@ -2677,9 +2686,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr"/>
-      <c r="D29" t="inlineStr"/>
-      <c r="E29" t="inlineStr"/>
     </row>
     <row r="30">
       <c r="A30" t="inlineStr">
@@ -2692,9 +2698,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C30" t="inlineStr"/>
-      <c r="D30" t="inlineStr"/>
-      <c r="E30" t="inlineStr"/>
     </row>
     <row r="31">
       <c r="A31" t="inlineStr">
@@ -2707,9 +2710,6 @@
           <t>합격</t>
         </is>
       </c>
-      <c r="C31" t="inlineStr"/>
-      <c r="D31" t="inlineStr"/>
-      <c r="E31" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>